<commit_message>
fix: WKF ProcessStem hierarchy - correct hasSIRManagerEmail propagation, rdfs:subClassOf default, scenario delete redirect, tree hideDraft filter
</commit_message>
<xml_diff>
--- a/wkf/WKF-ADMIN_MEDICACAO.xlsx
+++ b/wkf/WKF-ADMIN_MEDICACAO.xlsx
@@ -224,139 +224,132 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>STD</t>
+          <t>hasURI</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hasco:hasProcess</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Study ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Specific Aims</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Institution</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Principal Investigator</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>vstoi:hasLearningObjectives</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>vstoi:hasCriticalActions</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>vstoi:hasDebriefingFocus</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>https://pmsr.net/ont/WKF-ADMIN_MEDICACAO-20260811/STD/001</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hasURI</t>
+          <t>https://pmsr.net/ont/WKF-ADMIN_MEDICACAO-20260811/PROC/001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hasco:hasProcess</t>
+          <t>STD-ADMIN_MEDICACAO-001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Study ID</t>
+          <t>Administração Segura de Medicação</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Desenvolver competências clínicas de enfermagem.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Specific Aims</t>
+          <t>Segurança e qualidade dos cuidados.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Significance</t>
+          <t>pmsr:ORG174547834502838939</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Institution</t>
+          <t>pmsr:PER178793554744619146</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Principal Investigator</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Start Date</t>
+          <t>curator@reitoria.ucp.pt</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>End Date</t>
+          <t>Avaliação, segurança, comunicação.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>vstoi:hasLearningObjectives</t>
+          <t>Identificação correta, técnica segura, registo.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
-        <is>
-          <t>vstoi:hasCriticalActions</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>vstoi:hasDebriefingFocus</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://pmsr.net/ont/WKF-ADMIN_MEDICACAO-20260811/STD/001</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://pmsr.net/ont/WKF-ADMIN_MEDICACAO-20260811/PROC/001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>STD-ADMIN_MEDICACAO-001</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Administração Segura de Medicação</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Desenvolver competências clínicas de enfermagem.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Segurança e qualidade dos cuidados.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://pmsr.net/ont/ORG/ESS</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://pmsr.net/ont/PER/PI-001</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>equipa@pmsr.net</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Avaliação, segurança, comunicação.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Identificação correta, técnica segura, registo.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
         <is>
           <t>Tomada de decisão e melhoria contínua.</t>
         </is>

</xml_diff>